<commit_message>
update template removed prefilled numbers
</commit_message>
<xml_diff>
--- a/backend/Template/MonthlyReportTemplate.xlsx
+++ b/backend/Template/MonthlyReportTemplate.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
   <si>
     <t>WORLD MISSION PUBLICATIONS</t>
   </si>
@@ -57,9 +57,6 @@
     <t>Priest and Religious</t>
   </si>
   <si>
-    <t>Paid w/ Mass = 224</t>
-  </si>
-  <si>
     <t>Lay Persons</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t xml:space="preserve">Unencoded MP: </t>
   </si>
   <si>
-    <t>August (256), Sept (161)</t>
-  </si>
-  <si>
     <t>Total Paid Subscribers</t>
   </si>
   <si>
@@ -160,9 +154,6 @@
   </si>
   <si>
     <t>Date:</t>
-  </si>
-  <si>
-    <t>Oct 10, 2025</t>
   </si>
   <si>
     <t>Angel de Vera</t>
@@ -181,7 +172,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="13">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -260,14 +251,6 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
-    <font>
-      <b/>
-      <u/>
-      <sz val="10"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -480,7 +463,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -587,8 +570,6 @@
     <xf numFmtId="37" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -612,6 +593,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -919,7 +901,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1513,82 +1495,82 @@
   <sheetData>
     <row r="1" spans="1:11" ht="12.75" hidden="1" customHeight="1"/>
     <row r="2" spans="1:11">
-      <c r="A2" s="73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="73"/>
-      <c r="C2" s="73"/>
-      <c r="D2" s="73"/>
-      <c r="E2" s="73"/>
-      <c r="F2" s="73"/>
-      <c r="G2" s="73"/>
+      <c r="A2" s="71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="71"/>
+      <c r="F2" s="71"/>
+      <c r="G2" s="71"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="74" t="s">
+      <c r="A3" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="74"/>
-      <c r="C3" s="74"/>
-      <c r="D3" s="74"/>
-      <c r="E3" s="74"/>
-      <c r="F3" s="74"/>
-      <c r="G3" s="74"/>
+      <c r="B3" s="72"/>
+      <c r="C3" s="72"/>
+      <c r="D3" s="72"/>
+      <c r="E3" s="72"/>
+      <c r="F3" s="72"/>
+      <c r="G3" s="72"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="74" t="s">
+      <c r="A4" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="74"/>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
-      <c r="F4" s="74"/>
-      <c r="G4" s="74"/>
+      <c r="B4" s="72"/>
+      <c r="C4" s="72"/>
+      <c r="D4" s="72"/>
+      <c r="E4" s="72"/>
+      <c r="F4" s="72"/>
+      <c r="G4" s="72"/>
     </row>
     <row r="5" spans="1:11" ht="9.75" customHeight="1" thickBot="1">
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="18" customHeight="1" thickTop="1">
       <c r="A6" s="3"/>
-      <c r="B6" s="75" t="s">
+      <c r="B6" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="76"/>
-      <c r="D6" s="76"/>
-      <c r="E6" s="76"/>
-      <c r="F6" s="77"/>
+      <c r="C6" s="74"/>
+      <c r="D6" s="74"/>
+      <c r="E6" s="74"/>
+      <c r="F6" s="75"/>
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:11" ht="10.5" customHeight="1" thickBot="1">
-      <c r="B7" s="78"/>
-      <c r="C7" s="79"/>
-      <c r="D7" s="79"/>
-      <c r="E7" s="79"/>
-      <c r="F7" s="80"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="77"/>
+      <c r="D7" s="77"/>
+      <c r="E7" s="77"/>
+      <c r="F7" s="78"/>
       <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:11" ht="6" customHeight="1" thickTop="1">
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="22.5" customHeight="1">
-      <c r="A9" s="81" t="s">
+      <c r="A9" s="79" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="82"/>
-      <c r="C9" s="82"/>
-      <c r="D9" s="82"/>
-      <c r="E9" s="82"/>
-      <c r="F9" s="82"/>
-      <c r="G9" s="82"/>
+      <c r="B9" s="80"/>
+      <c r="C9" s="80"/>
+      <c r="D9" s="80"/>
+      <c r="E9" s="80"/>
+      <c r="F9" s="80"/>
+      <c r="G9" s="80"/>
     </row>
     <row r="10" spans="1:11" ht="2.25" hidden="1" customHeight="1">
-      <c r="A10" s="82"/>
-      <c r="B10" s="82"/>
-      <c r="C10" s="82"/>
-      <c r="D10" s="82"/>
-      <c r="E10" s="82"/>
-      <c r="F10" s="82"/>
-      <c r="G10" s="82"/>
+      <c r="A10" s="80"/>
+      <c r="B10" s="80"/>
+      <c r="C10" s="80"/>
+      <c r="D10" s="80"/>
+      <c r="E10" s="80"/>
+      <c r="F10" s="80"/>
+      <c r="G10" s="80"/>
     </row>
     <row r="11" spans="1:11">
       <c r="G11" s="5" t="s">
@@ -1607,9 +1589,7 @@
       <c r="F13" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G13" s="67">
-        <v>4850</v>
-      </c>
+      <c r="G13" s="67"/>
     </row>
     <row r="14" spans="1:11" ht="6.75" customHeight="1">
       <c r="A14" s="5"/>
@@ -1648,69 +1628,51 @@
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="17"/>
-      <c r="D17" s="18" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" s="19">
-        <v>253</v>
-      </c>
-      <c r="F17" s="20">
-        <v>41</v>
-      </c>
+      <c r="D17" s="18"/>
+      <c r="E17" s="19"/>
+      <c r="F17" s="20"/>
       <c r="G17" s="19">
-        <f t="shared" ref="G17:G22" si="0">SUM(E17:F17)</f>
-        <v>294</v>
+        <f t="shared" ref="G17:G21" si="0">SUM(E17:F17)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="21" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B18" s="22"/>
       <c r="C18" s="22"/>
       <c r="D18" s="23"/>
-      <c r="E18" s="19">
-        <v>2726</v>
-      </c>
-      <c r="F18" s="20">
-        <v>12</v>
-      </c>
+      <c r="E18" s="19"/>
+      <c r="F18" s="20"/>
       <c r="G18" s="19">
         <f t="shared" si="0"/>
-        <v>2738</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="21" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B19" s="22"/>
       <c r="C19" s="22"/>
       <c r="D19" s="24"/>
-      <c r="E19" s="19">
-        <v>7</v>
-      </c>
-      <c r="F19" s="20">
-        <v>5</v>
-      </c>
+      <c r="E19" s="19"/>
+      <c r="F19" s="20"/>
       <c r="G19" s="19">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B20" s="22"/>
       <c r="C20" s="22"/>
       <c r="D20" s="24"/>
-      <c r="E20" s="19">
-        <v>0</v>
-      </c>
-      <c r="F20" s="25">
-        <v>0</v>
-      </c>
+      <c r="E20" s="19"/>
+      <c r="F20" s="25"/>
       <c r="G20" s="19">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1719,60 +1681,50 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B21" s="22"/>
       <c r="C21" s="22"/>
       <c r="D21" s="24"/>
-      <c r="E21" s="19">
-        <v>137</v>
-      </c>
-      <c r="F21" s="25">
-        <v>3</v>
-      </c>
+      <c r="E21" s="19"/>
+      <c r="F21" s="25"/>
       <c r="G21" s="19">
         <f t="shared" si="0"/>
-        <v>140</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="B22" s="72" t="s">
-        <v>17</v>
-      </c>
-      <c r="C22" s="72"/>
-      <c r="D22" s="72"/>
-      <c r="E22" s="31">
-        <v>417</v>
-      </c>
-      <c r="F22" s="27">
-        <v>0</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="B22" s="70"/>
+      <c r="C22" s="70"/>
+      <c r="D22" s="70"/>
+      <c r="E22" s="31"/>
+      <c r="F22" s="27"/>
       <c r="G22" s="19">
         <f>SUM(E22:F22)</f>
-        <v>417</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:9" s="35" customFormat="1">
       <c r="A23" s="28" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B23" s="29"/>
       <c r="C23" s="29"/>
       <c r="D23" s="30"/>
       <c r="E23" s="31">
         <f>SUM(E17:E22)</f>
-        <v>3540</v>
+        <v>0</v>
       </c>
       <c r="F23" s="32">
         <f>SUM(F17:F22)</f>
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="G23" s="33">
         <f>SUM(G17:G22)</f>
-        <v>3601</v>
+        <v>0</v>
       </c>
       <c r="H23" s="34"/>
       <c r="I23" s="34"/>
@@ -1787,45 +1739,37 @@
     </row>
     <row r="25" spans="1:9" ht="12.75" customHeight="1">
       <c r="A25" s="38" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B25" s="35"/>
       <c r="C25" s="35"/>
       <c r="D25" s="39"/>
       <c r="E25" s="40"/>
       <c r="F25" s="41"/>
-      <c r="G25" s="19">
-        <v>118</v>
-      </c>
+      <c r="G25" s="19"/>
     </row>
     <row r="26" spans="1:9" ht="12.75" customHeight="1">
       <c r="A26" s="38" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
       <c r="D26" s="39"/>
       <c r="E26" s="42"/>
       <c r="F26" s="41"/>
-      <c r="G26" s="19">
-        <v>35</v>
-      </c>
+      <c r="G26" s="19"/>
     </row>
     <row r="27" spans="1:9" ht="12.75" customHeight="1">
       <c r="A27" s="38" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B27" s="35"/>
       <c r="C27" s="43"/>
-      <c r="D27" s="68">
-        <v>512</v>
-      </c>
+      <c r="D27" s="68"/>
       <c r="E27" s="42" t="s">
-        <v>22</v>
-      </c>
-      <c r="F27" s="69">
-        <v>2</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F27" s="69"/>
       <c r="G27" s="19"/>
       <c r="H27" s="44"/>
     </row>
@@ -1837,8 +1781,8 @@
       <c r="G28" s="19"/>
     </row>
     <row r="29" spans="1:9">
-      <c r="A29" s="70" t="s">
-        <v>23</v>
+      <c r="A29" s="81" t="s">
+        <v>21</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1849,53 +1793,41 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="48"/>
       <c r="D30" s="23"/>
-      <c r="E30" s="40">
-        <v>11</v>
-      </c>
-      <c r="F30" s="20">
-        <v>0</v>
-      </c>
+      <c r="E30" s="40"/>
+      <c r="F30" s="20"/>
       <c r="G30" s="19">
         <f>SUM(E30:F30)</f>
-        <v>11</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B31" s="22"/>
       <c r="C31" s="49"/>
       <c r="D31" s="24"/>
-      <c r="E31" s="40">
-        <v>71</v>
-      </c>
-      <c r="F31" s="20">
-        <v>0</v>
-      </c>
+      <c r="E31" s="40"/>
+      <c r="F31" s="20"/>
       <c r="G31" s="19">
         <f>SUM(E31:F31)</f>
-        <v>71</v>
+        <v>0</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="49"/>
       <c r="D32" s="24"/>
-      <c r="E32" s="50">
-        <v>0</v>
-      </c>
-      <c r="F32" s="51">
-        <v>0</v>
-      </c>
+      <c r="E32" s="50"/>
+      <c r="F32" s="51"/>
       <c r="G32" s="19">
         <f>SUM(E32:F32)</f>
         <v>0</v>
@@ -1903,17 +1835,13 @@
     </row>
     <row r="33" spans="1:15" hidden="1">
       <c r="A33" s="21" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B33" s="22"/>
       <c r="C33" s="49"/>
       <c r="D33" s="24"/>
-      <c r="E33" s="26">
-        <v>0</v>
-      </c>
-      <c r="F33" s="51">
-        <v>0</v>
-      </c>
+      <c r="E33" s="26"/>
+      <c r="F33" s="51"/>
       <c r="G33" s="19">
         <f>SUM(E33:F33)</f>
         <v>0</v>
@@ -1921,14 +1849,14 @@
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="28" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B34" s="29"/>
       <c r="C34" s="29"/>
       <c r="D34" s="52"/>
       <c r="E34" s="31">
         <f>SUM(E30:E33)</f>
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="F34" s="32">
         <f>SUM(F30:F33)</f>
@@ -1936,7 +1864,7 @@
       </c>
       <c r="G34" s="37">
         <f>SUM(G30:G33)</f>
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="H34" s="44"/>
       <c r="I34" s="44"/>
@@ -1954,22 +1882,22 @@
     </row>
     <row r="36" spans="1:15" s="35" customFormat="1">
       <c r="A36" s="29" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29"/>
       <c r="D36" s="52"/>
       <c r="E36" s="31">
         <f>SUM(E23,E34)</f>
-        <v>3622</v>
+        <v>0</v>
       </c>
       <c r="F36" s="31">
         <f>SUM(F23,F34)</f>
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="G36" s="31">
         <f>SUM(G23,G34)</f>
-        <v>3683</v>
+        <v>0</v>
       </c>
       <c r="H36" s="34"/>
       <c r="I36" s="34"/>
@@ -1982,8 +1910,8 @@
       <c r="G37" s="19"/>
     </row>
     <row r="38" spans="1:15">
-      <c r="A38" s="70" t="s">
-        <v>30</v>
+      <c r="A38" s="81" t="s">
+        <v>28</v>
       </c>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
@@ -1994,53 +1922,41 @@
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="48"/>
       <c r="D39" s="23"/>
-      <c r="E39" s="40">
-        <v>288</v>
-      </c>
-      <c r="F39" s="20">
-        <v>0</v>
-      </c>
+      <c r="E39" s="40"/>
+      <c r="F39" s="20"/>
       <c r="G39" s="19">
         <f>SUM(E39:F39)</f>
-        <v>288</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="21" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B40" s="22"/>
       <c r="C40" s="49"/>
       <c r="D40" s="24"/>
-      <c r="E40" s="40">
-        <v>20</v>
-      </c>
-      <c r="F40" s="25">
-        <v>0</v>
-      </c>
+      <c r="E40" s="40"/>
+      <c r="F40" s="25"/>
       <c r="G40" s="19">
         <f>SUM(E40:F40)</f>
-        <v>20</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="21" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B41" s="22"/>
       <c r="C41" s="49"/>
       <c r="D41" s="24"/>
-      <c r="E41" s="50">
-        <v>0</v>
-      </c>
-      <c r="F41" s="27">
-        <v>0</v>
-      </c>
+      <c r="E41" s="50"/>
+      <c r="F41" s="27"/>
       <c r="G41" s="19">
         <f>SUM(E41:F41)</f>
         <v>0</v>
@@ -2048,14 +1964,14 @@
     </row>
     <row r="42" spans="1:15" s="35" customFormat="1">
       <c r="A42" s="28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B42" s="29"/>
       <c r="C42" s="29"/>
       <c r="D42" s="30"/>
       <c r="E42" s="31">
         <f>SUM(E39:E41)</f>
-        <v>308</v>
+        <v>0</v>
       </c>
       <c r="F42" s="54">
         <f>SUM(F39:F41)</f>
@@ -2063,7 +1979,7 @@
       </c>
       <c r="G42" s="31">
         <f>SUM(G39:G41)</f>
-        <v>308</v>
+        <v>0</v>
       </c>
       <c r="H42" s="34"/>
       <c r="I42" s="34"/>
@@ -2077,7 +1993,7 @@
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="10" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
@@ -2088,95 +2004,79 @@
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="15" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
       <c r="D45" s="23"/>
-      <c r="E45" s="19">
-        <v>124</v>
-      </c>
-      <c r="F45" s="20">
-        <v>0</v>
-      </c>
+      <c r="E45" s="19"/>
+      <c r="F45" s="20"/>
       <c r="G45" s="19">
         <f>SUM(E45:F45)</f>
-        <v>124</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B46" s="22"/>
       <c r="C46" s="22"/>
       <c r="D46" s="24"/>
-      <c r="E46" s="19">
-        <v>120</v>
-      </c>
-      <c r="F46" s="20">
-        <v>65</v>
-      </c>
+      <c r="E46" s="19"/>
+      <c r="F46" s="20"/>
       <c r="G46" s="19">
         <f>SUM(E46:F46)</f>
-        <v>185</v>
+        <v>0</v>
       </c>
       <c r="O46" s="39"/>
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="21" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B47" s="22"/>
       <c r="C47" s="22"/>
       <c r="D47" s="24"/>
-      <c r="E47" s="19">
-        <v>2</v>
-      </c>
-      <c r="F47" s="20">
-        <v>6</v>
-      </c>
+      <c r="E47" s="19"/>
+      <c r="F47" s="20"/>
       <c r="G47" s="19">
         <f>SUM(E47:F47)</f>
-        <v>8</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:15">
-      <c r="A48" s="71" t="s">
-        <v>39</v>
+      <c r="A48" s="21" t="s">
+        <v>37</v>
       </c>
       <c r="B48" s="22"/>
       <c r="C48" s="22"/>
       <c r="D48" s="24"/>
-      <c r="E48" s="50">
-        <v>10</v>
-      </c>
-      <c r="F48" s="27">
-        <v>0</v>
-      </c>
+      <c r="E48" s="50"/>
+      <c r="F48" s="27"/>
       <c r="G48" s="19">
         <f>SUM(E48:F48)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49" spans="1:9" s="35" customFormat="1">
       <c r="A49" s="28" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B49" s="29"/>
       <c r="C49" s="29"/>
       <c r="D49" s="30"/>
       <c r="E49" s="31">
         <f>SUM(E45:E48)</f>
-        <v>256</v>
+        <v>0</v>
       </c>
       <c r="F49" s="32">
         <f>SUM(F45:F48)</f>
-        <v>71</v>
+        <v>0</v>
       </c>
       <c r="G49" s="33">
         <f>SUM(G45:G48)</f>
-        <v>327</v>
+        <v>0</v>
       </c>
       <c r="H49" s="2"/>
       <c r="I49" s="34"/>
@@ -2191,36 +2091,34 @@
     </row>
     <row r="51" spans="1:9">
       <c r="A51" s="35" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B51" s="35"/>
       <c r="C51" s="35"/>
       <c r="D51" s="39"/>
-      <c r="E51" s="55">
-        <v>56</v>
-      </c>
+      <c r="E51" s="55"/>
       <c r="F51" s="55"/>
       <c r="G51" s="56"/>
       <c r="H51" s="44"/>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="29" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B52" s="29"/>
       <c r="C52" s="29"/>
       <c r="D52" s="52"/>
       <c r="E52" s="57">
         <f>SUM(E36,E42,E49,E51)</f>
-        <v>4242</v>
+        <v>0</v>
       </c>
       <c r="F52" s="57">
         <f>SUM(F51,F49,F36)</f>
-        <v>132</v>
+        <v>0</v>
       </c>
       <c r="G52" s="57">
         <f>SUM(G36,G42,G49)+E51</f>
-        <v>4374</v>
+        <v>0</v>
       </c>
       <c r="H52" s="2"/>
     </row>
@@ -2240,11 +2138,11 @@
       <c r="D54" s="58"/>
       <c r="E54" s="59"/>
       <c r="F54" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G54" s="57">
         <f>G13-G52</f>
-        <v>476</v>
+        <v>0</v>
       </c>
       <c r="I54" s="35"/>
     </row>
@@ -2258,28 +2156,26 @@
     <row r="56" spans="1:9" ht="6.75" customHeight="1"/>
     <row r="57" spans="1:9">
       <c r="E57" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="I57" s="62"/>
     </row>
     <row r="59" spans="1:9" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:9">
       <c r="A60" s="63" t="s">
-        <v>45</v>
-      </c>
-      <c r="B60" s="64" t="s">
-        <v>46</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="B60" s="64"/>
       <c r="E60" s="1" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="61" spans="1:9">
       <c r="B61" s="65" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="62" spans="1:9">

</xml_diff>

<commit_message>
updated template to match the users request
</commit_message>
<xml_diff>
--- a/backend/Template/MonthlyReportTemplate.xlsx
+++ b/backend/Template/MonthlyReportTemplate.xlsx
@@ -78,12 +78,6 @@
     <t>NEW SUBSCRIBERS for the month</t>
   </si>
   <si>
-    <t>RENEWALS during the month of  SEPT 2025</t>
-  </si>
-  <si>
-    <t>DUE FOR RENEWAL for the mo. of SEPT 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve">Renewed = </t>
   </si>
   <si>
@@ -163,6 +157,12 @@
   </si>
   <si>
     <t>Circulation Officer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RENEWALS during the month of  </t>
+  </si>
+  <si>
+    <t>DUE FOR RENEWAL for the month of</t>
   </si>
 </sst>
 </file>
@@ -570,6 +570,7 @@
     <xf numFmtId="37" fontId="11" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -593,7 +594,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -901,7 +901,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -915,7 +915,7 @@
   <dimension ref="A1:O62"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
-    <col min="1" max="1" width="18.140625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="17.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="28.7109375" style="1" customWidth="1"/>
     <col min="3" max="3" width="6.85546875" style="1" hidden="1" customWidth="1"/>
     <col min="4" max="4" width="13.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -1495,82 +1495,82 @@
   <sheetData>
     <row r="1" spans="1:11" ht="12.75" hidden="1" customHeight="1"/>
     <row r="2" spans="1:11">
-      <c r="A2" s="71" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="71"/>
+      <c r="A2" s="72" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="72"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
     </row>
     <row r="3" spans="1:11">
-      <c r="A3" s="72" t="s">
+      <c r="A3" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="72"/>
-      <c r="C3" s="72"/>
-      <c r="D3" s="72"/>
-      <c r="E3" s="72"/>
-      <c r="F3" s="72"/>
-      <c r="G3" s="72"/>
+      <c r="B3" s="73"/>
+      <c r="C3" s="73"/>
+      <c r="D3" s="73"/>
+      <c r="E3" s="73"/>
+      <c r="F3" s="73"/>
+      <c r="G3" s="73"/>
     </row>
     <row r="4" spans="1:11">
-      <c r="A4" s="72" t="s">
+      <c r="A4" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="72"/>
-      <c r="C4" s="72"/>
-      <c r="D4" s="72"/>
-      <c r="E4" s="72"/>
-      <c r="F4" s="72"/>
-      <c r="G4" s="72"/>
+      <c r="B4" s="73"/>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="73"/>
+      <c r="F4" s="73"/>
+      <c r="G4" s="73"/>
     </row>
     <row r="5" spans="1:11" ht="9.75" customHeight="1" thickBot="1">
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:11" ht="18" customHeight="1" thickTop="1">
       <c r="A6" s="3"/>
-      <c r="B6" s="73" t="s">
+      <c r="B6" s="74" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="74"/>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-      <c r="F6" s="75"/>
+      <c r="C6" s="75"/>
+      <c r="D6" s="75"/>
+      <c r="E6" s="75"/>
+      <c r="F6" s="76"/>
       <c r="G6" s="4"/>
     </row>
     <row r="7" spans="1:11" ht="10.5" customHeight="1" thickBot="1">
-      <c r="B7" s="76"/>
-      <c r="C7" s="77"/>
-      <c r="D7" s="77"/>
-      <c r="E7" s="77"/>
-      <c r="F7" s="78"/>
+      <c r="B7" s="77"/>
+      <c r="C7" s="78"/>
+      <c r="D7" s="78"/>
+      <c r="E7" s="78"/>
+      <c r="F7" s="79"/>
       <c r="G7" s="4"/>
     </row>
     <row r="8" spans="1:11" ht="6" customHeight="1" thickTop="1">
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:11" ht="22.5" customHeight="1">
-      <c r="A9" s="79" t="s">
+      <c r="A9" s="80" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="80"/>
-      <c r="C9" s="80"/>
-      <c r="D9" s="80"/>
-      <c r="E9" s="80"/>
-      <c r="F9" s="80"/>
-      <c r="G9" s="80"/>
+      <c r="B9" s="81"/>
+      <c r="C9" s="81"/>
+      <c r="D9" s="81"/>
+      <c r="E9" s="81"/>
+      <c r="F9" s="81"/>
+      <c r="G9" s="81"/>
     </row>
     <row r="10" spans="1:11" ht="2.25" hidden="1" customHeight="1">
-      <c r="A10" s="80"/>
-      <c r="B10" s="80"/>
-      <c r="C10" s="80"/>
-      <c r="D10" s="80"/>
-      <c r="E10" s="80"/>
-      <c r="F10" s="80"/>
-      <c r="G10" s="80"/>
+      <c r="A10" s="81"/>
+      <c r="B10" s="81"/>
+      <c r="C10" s="81"/>
+      <c r="D10" s="81"/>
+      <c r="E10" s="81"/>
+      <c r="F10" s="81"/>
+      <c r="G10" s="81"/>
     </row>
     <row r="11" spans="1:11">
       <c r="G11" s="5" t="s">
@@ -1697,9 +1697,9 @@
       <c r="A22" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="B22" s="70"/>
-      <c r="C22" s="70"/>
-      <c r="D22" s="70"/>
+      <c r="B22" s="71"/>
+      <c r="C22" s="71"/>
+      <c r="D22" s="71"/>
       <c r="E22" s="31"/>
       <c r="F22" s="27"/>
       <c r="G22" s="19">
@@ -1750,7 +1750,7 @@
     </row>
     <row r="26" spans="1:9" ht="12.75" customHeight="1">
       <c r="A26" s="38" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="B26" s="35"/>
       <c r="C26" s="35"/>
@@ -1761,13 +1761,13 @@
     </row>
     <row r="27" spans="1:9" ht="12.75" customHeight="1">
       <c r="A27" s="38" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="B27" s="35"/>
       <c r="C27" s="43"/>
       <c r="D27" s="68"/>
       <c r="E27" s="42" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F27" s="69"/>
       <c r="G27" s="19"/>
@@ -1781,8 +1781,8 @@
       <c r="G28" s="19"/>
     </row>
     <row r="29" spans="1:9">
-      <c r="A29" s="81" t="s">
-        <v>21</v>
+      <c r="A29" s="70" t="s">
+        <v>19</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -1793,7 +1793,7 @@
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="48"/>
@@ -1807,7 +1807,7 @@
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="21" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B31" s="22"/>
       <c r="C31" s="49"/>
@@ -1821,7 +1821,7 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="49"/>
@@ -1835,7 +1835,7 @@
     </row>
     <row r="33" spans="1:15" hidden="1">
       <c r="A33" s="21" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B33" s="22"/>
       <c r="C33" s="49"/>
@@ -1849,7 +1849,7 @@
     </row>
     <row r="34" spans="1:15">
       <c r="A34" s="28" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B34" s="29"/>
       <c r="C34" s="29"/>
@@ -1882,7 +1882,7 @@
     </row>
     <row r="36" spans="1:15" s="35" customFormat="1">
       <c r="A36" s="29" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B36" s="29"/>
       <c r="C36" s="29"/>
@@ -1910,8 +1910,8 @@
       <c r="G37" s="19"/>
     </row>
     <row r="38" spans="1:15">
-      <c r="A38" s="81" t="s">
-        <v>28</v>
+      <c r="A38" s="70" t="s">
+        <v>26</v>
       </c>
       <c r="B38" s="11"/>
       <c r="C38" s="11"/>
@@ -1922,7 +1922,7 @@
     </row>
     <row r="39" spans="1:15">
       <c r="A39" s="15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="48"/>
@@ -1936,7 +1936,7 @@
     </row>
     <row r="40" spans="1:15">
       <c r="A40" s="21" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B40" s="22"/>
       <c r="C40" s="49"/>
@@ -1950,7 +1950,7 @@
     </row>
     <row r="41" spans="1:15">
       <c r="A41" s="21" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B41" s="22"/>
       <c r="C41" s="49"/>
@@ -1964,7 +1964,7 @@
     </row>
     <row r="42" spans="1:15" s="35" customFormat="1">
       <c r="A42" s="28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B42" s="29"/>
       <c r="C42" s="29"/>
@@ -1993,7 +1993,7 @@
     </row>
     <row r="44" spans="1:15">
       <c r="A44" s="10" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B44" s="11"/>
       <c r="C44" s="11"/>
@@ -2004,7 +2004,7 @@
     </row>
     <row r="45" spans="1:15">
       <c r="A45" s="15" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
@@ -2018,7 +2018,7 @@
     </row>
     <row r="46" spans="1:15">
       <c r="A46" s="21" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B46" s="22"/>
       <c r="C46" s="22"/>
@@ -2033,7 +2033,7 @@
     </row>
     <row r="47" spans="1:15">
       <c r="A47" s="21" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B47" s="22"/>
       <c r="C47" s="22"/>
@@ -2047,7 +2047,7 @@
     </row>
     <row r="48" spans="1:15">
       <c r="A48" s="21" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B48" s="22"/>
       <c r="C48" s="22"/>
@@ -2061,7 +2061,7 @@
     </row>
     <row r="49" spans="1:9" s="35" customFormat="1">
       <c r="A49" s="28" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B49" s="29"/>
       <c r="C49" s="29"/>
@@ -2091,7 +2091,7 @@
     </row>
     <row r="51" spans="1:9">
       <c r="A51" s="35" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B51" s="35"/>
       <c r="C51" s="35"/>
@@ -2103,7 +2103,7 @@
     </row>
     <row r="52" spans="1:9">
       <c r="A52" s="29" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B52" s="29"/>
       <c r="C52" s="29"/>
@@ -2138,7 +2138,7 @@
       <c r="D54" s="58"/>
       <c r="E54" s="59"/>
       <c r="F54" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G54" s="57">
         <f>G13-G52</f>
@@ -2156,26 +2156,26 @@
     <row r="56" spans="1:9" ht="6.75" customHeight="1"/>
     <row r="57" spans="1:9">
       <c r="E57" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="I57" s="62"/>
     </row>
     <row r="59" spans="1:9" ht="14.25" customHeight="1"/>
     <row r="60" spans="1:9">
       <c r="A60" s="63" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B60" s="64"/>
       <c r="E60" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="61" spans="1:9">
       <c r="B61" s="65" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="62" spans="1:9">

</xml_diff>